<commit_message>
Apply user taxonomy corrections (162 edits): new 'Yemek Seti' type, name standardization
- taksonomi.xlsx: 96 name + 64 type corrections from user review (sets -> 'Yemek Seti',
  ESTETIK LUX -> LUX KAŞIK/BIÇAK, PRIZMA KAP reorder, etc)
- dashboard.html: add EN translations for 13 product types (Kase, Köpük Tepsi, İçecek
  Bardağı, Yemek Kutusu, etc) to KAT_EN + TIP_EN
- product_en.json: EN names for renamed products (X-PC SET, PRISM CONTAINER, etc)
- Rebuilt: 203 products (more consolidation), $6.50M, all types translated

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RoehW9ESGDK2XkibhR7KNP
</commit_message>
<xml_diff>
--- a/data/taksonomi.xlsx
+++ b/data/taksonomi.xlsx
@@ -674,7 +674,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>PRIZMA KAP 120 CC</t>
+          <t>120 CC PRIZMA KAP</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>PRIZMA KAP 60 CC</t>
+          <t>60 CC PRIZMA KAP</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
@@ -1412,7 +1412,7 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>PRIZMA KAP 200 CC</t>
+          <t>200 CC PRIZMA KAP</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>DIAMOND YEMEK SETİ 4'lü</t>
+          <t>DIAMOND 4LÜ SET</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>PREMIUM YEMEK SETİ 4'lü</t>
+          <t>PREMIUM 4LÜ SET</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
@@ -2119,7 +2119,7 @@
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>DIAMOND YEMEK SETİ 3'lü</t>
+          <t>DIAMOND 3LÜ SET</t>
         </is>
       </c>
       <c r="D71" s="8" t="inlineStr">
@@ -3431,7 +3431,7 @@
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F71" s="8" t="inlineStr">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>DIAMOND YEMEK SETİ 4'lü</t>
+          <t>DIAMOND 4LÜ SET</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
@@ -3636,7 +3636,7 @@
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F76" s="7" t="inlineStr">
@@ -3667,7 +3667,7 @@
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>DIAMOND YEMEK SETİ 3'lü</t>
+          <t>DIAMOND 3LÜ SET</t>
         </is>
       </c>
       <c r="D77" s="8" t="inlineStr">
@@ -3677,7 +3677,7 @@
       </c>
       <c r="E77" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F77" s="8" t="inlineStr">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>PREMIUM SET 4'lü</t>
+          <t>PREMIUM 4LÜ SET</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F78" s="7" t="inlineStr">
@@ -3749,7 +3749,7 @@
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>PREMIUM YEMEK SETİ 6'lü</t>
+          <t>PREMIUM 6LI SET</t>
         </is>
       </c>
       <c r="D79" s="8" t="inlineStr">
@@ -3759,7 +3759,7 @@
       </c>
       <c r="E79" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F79" s="8" t="inlineStr">
@@ -4036,7 +4036,7 @@
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>PREMIUM YEMEK SETİ 4'lü</t>
+          <t>PREMIUM 4LÜ SET</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
@@ -4046,7 +4046,7 @@
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F86" s="7" t="inlineStr">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>PREMIUM YEMEK SET 3'lü</t>
+          <t>PREMIUM 3LÜ SET</t>
         </is>
       </c>
       <c r="D87" s="8" t="inlineStr">
@@ -4087,7 +4087,7 @@
       </c>
       <c r="E87" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F87" s="8" t="inlineStr">
@@ -4118,7 +4118,7 @@
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>PREMIUM YEMEK SET 3'lü</t>
+          <t>PREMIUM 3LÜ SET</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
@@ -4128,7 +4128,7 @@
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F88" s="7" t="inlineStr">
@@ -4282,7 +4282,7 @@
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>ELITE YEMEK SETİ 4'lü</t>
+          <t>ELITE 4LÜ SET</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
@@ -4292,7 +4292,7 @@
       </c>
       <c r="E92" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F92" s="7" t="inlineStr">
@@ -4446,7 +4446,7 @@
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>ELITE YEMEK SETİ 3'lü</t>
+          <t>ELITE 3LÜ SET</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
@@ -4456,7 +4456,7 @@
       </c>
       <c r="E96" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F96" s="7" t="inlineStr">
@@ -4579,7 +4579,7 @@
       </c>
       <c r="E99" s="8" t="inlineStr">
         <is>
-          <t>Çatal</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F99" s="8" t="inlineStr">
@@ -4856,7 +4856,7 @@
       </c>
       <c r="C106" s="6" t="inlineStr">
         <is>
-          <t>EKO YEMEK SETİ 4'lü</t>
+          <t>EKO 4LÜ SET</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
@@ -4866,7 +4866,7 @@
       </c>
       <c r="E106" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F106" s="7" t="inlineStr">
@@ -5020,7 +5020,7 @@
       </c>
       <c r="C110" s="6" t="inlineStr">
         <is>
-          <t>YEMEK SETi 4'lü</t>
+          <t>PREMIUM 4LÜ SET</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
@@ -5030,7 +5030,7 @@
       </c>
       <c r="E110" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F110" s="7" t="inlineStr">
@@ -5102,7 +5102,7 @@
       </c>
       <c r="C112" s="6" t="inlineStr">
         <is>
-          <t>30 CC (1 OZ) KAPAKLI SOS KABI</t>
+          <t>1 OZ (30 CC) SOS KABI</t>
         </is>
       </c>
       <c r="D112" s="7" t="inlineStr">
@@ -5143,7 +5143,7 @@
       </c>
       <c r="C113" s="6" t="inlineStr">
         <is>
-          <t>PREMIUM SET 3'lü</t>
+          <t>PREMIUM 3LÜ SET</t>
         </is>
       </c>
       <c r="D113" s="8" t="inlineStr">
@@ -5153,7 +5153,7 @@
       </c>
       <c r="E113" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F113" s="8" t="inlineStr">
@@ -5635,7 +5635,7 @@
       </c>
       <c r="C125" s="6" t="inlineStr">
         <is>
-          <t>PREMIUM YEMEK SETİ 3'lü</t>
+          <t>PREMIUM 3LÜ SET</t>
         </is>
       </c>
       <c r="D125" s="8" t="inlineStr">
@@ -5645,7 +5645,7 @@
       </c>
       <c r="E125" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F125" s="8" t="inlineStr">
@@ -5676,7 +5676,7 @@
       </c>
       <c r="C126" s="6" t="inlineStr">
         <is>
-          <t>DIAMOND YEMEK SETİ 3'lü</t>
+          <t>DIAMOND 3LÜ SET</t>
         </is>
       </c>
       <c r="D126" s="7" t="inlineStr">
@@ -5686,7 +5686,7 @@
       </c>
       <c r="E126" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F126" s="7" t="inlineStr">
@@ -5799,7 +5799,7 @@
       </c>
       <c r="C129" s="6" t="inlineStr">
         <is>
-          <t>LÜKS CİPS ÇATALI</t>
+          <t>LUX CİPS ÇATALI</t>
         </is>
       </c>
       <c r="D129" s="8" t="inlineStr">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="C133" s="6" t="inlineStr">
         <is>
-          <t>ÇATAL PLATINUM TEKLİ SET</t>
+          <t>PLATINUM ÇATAL TEKLİ SET</t>
         </is>
       </c>
       <c r="D133" s="8" t="inlineStr">
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E133" s="8" t="inlineStr">
         <is>
-          <t>Çatal</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F133" s="8" t="inlineStr">
@@ -6055,7 +6055,7 @@
       </c>
       <c r="E135" s="8" t="inlineStr">
         <is>
-          <t>Dondurma Kaşığı</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F135" s="8" t="inlineStr">
@@ -6291,7 +6291,7 @@
       </c>
       <c r="C141" s="6" t="inlineStr">
         <is>
-          <t>SET 6'lü Ç+K</t>
+          <t>LUX 6LI SET</t>
         </is>
       </c>
       <c r="D141" s="8" t="inlineStr">
@@ -6301,7 +6301,7 @@
       </c>
       <c r="E141" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F141" s="8" t="inlineStr">
@@ -6496,7 +6496,7 @@
       </c>
       <c r="C146" s="6" t="inlineStr">
         <is>
-          <t>PREMİUM SET 3'lü ÇATAL BIÇAK PEÇETE</t>
+          <t>PREMIUM 3LÜ SET</t>
         </is>
       </c>
       <c r="D146" s="7" t="inlineStr">
@@ -6506,7 +6506,7 @@
       </c>
       <c r="E146" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F146" s="7" t="inlineStr">
@@ -7275,7 +7275,7 @@
       </c>
       <c r="C165" s="6" t="inlineStr">
         <is>
-          <t>PLA YEMEK SETİ</t>
+          <t>PLA SET</t>
         </is>
       </c>
       <c r="D165" s="8" t="inlineStr">
@@ -7285,7 +7285,7 @@
       </c>
       <c r="E165" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F165" s="8" t="inlineStr">
@@ -7398,7 +7398,7 @@
       </c>
       <c r="C168" s="6" t="inlineStr">
         <is>
-          <t>PREMIUM YEMEK SETİ 3'lü</t>
+          <t>PREMIUM 3LÜ SET</t>
         </is>
       </c>
       <c r="D168" s="7" t="inlineStr">
@@ -7408,7 +7408,7 @@
       </c>
       <c r="E168" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F168" s="7" t="inlineStr">
@@ -7439,7 +7439,7 @@
       </c>
       <c r="C169" s="6" t="inlineStr">
         <is>
-          <t>EKO YEMEK SETİ 3'lü</t>
+          <t>EKO 3LÜ SET</t>
         </is>
       </c>
       <c r="D169" s="8" t="inlineStr">
@@ -7449,7 +7449,7 @@
       </c>
       <c r="E169" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F169" s="8" t="inlineStr">
@@ -7562,7 +7562,7 @@
       </c>
       <c r="C172" s="6" t="inlineStr">
         <is>
-          <t>PREMIUM YEMEK SETİ 2'lü</t>
+          <t>PREMIUM 2Lİ SET</t>
         </is>
       </c>
       <c r="D172" s="7" t="inlineStr">
@@ -7572,7 +7572,7 @@
       </c>
       <c r="E172" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F172" s="7" t="inlineStr">
@@ -7603,7 +7603,7 @@
       </c>
       <c r="C173" s="6" t="inlineStr">
         <is>
-          <t>EKO YEMEK SETİ 3'lü</t>
+          <t>EKO 3LÜ SET</t>
         </is>
       </c>
       <c r="D173" s="8" t="inlineStr">
@@ -7613,7 +7613,7 @@
       </c>
       <c r="E173" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F173" s="8" t="inlineStr">
@@ -7813,7 +7813,7 @@
       </c>
       <c r="D178" s="8" t="inlineStr">
         <is>
-          <t>XPS</t>
+          <t>PS</t>
         </is>
       </c>
       <c r="E178" s="7" t="inlineStr">
@@ -7823,7 +7823,7 @@
       </c>
       <c r="F178" s="8" t="inlineStr">
         <is>
-          <t>Foam/XPS</t>
+          <t>Standart</t>
         </is>
       </c>
       <c r="G178" s="7" t="inlineStr">
@@ -7849,7 +7849,7 @@
       </c>
       <c r="C179" s="6" t="inlineStr">
         <is>
-          <t>PREMIUM YEMEK SETİ 4'lü</t>
+          <t>PREMIUM 4LÜ SET</t>
         </is>
       </c>
       <c r="D179" s="8" t="inlineStr">
@@ -7859,7 +7859,7 @@
       </c>
       <c r="E179" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F179" s="8" t="inlineStr">
@@ -7890,7 +7890,7 @@
       </c>
       <c r="C180" s="6" t="inlineStr">
         <is>
-          <t>ÇATAL PLATINUM TEKLİ SET</t>
+          <t>PLATINUM ÇATAL TEKLİ SET</t>
         </is>
       </c>
       <c r="D180" s="7" t="inlineStr">
@@ -7900,7 +7900,7 @@
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
-          <t>Çatal</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F180" s="7" t="inlineStr">
@@ -8187,7 +8187,7 @@
       </c>
       <c r="E187" s="8" t="inlineStr">
         <is>
-          <t>Kaşık</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F187" s="8" t="inlineStr">
@@ -8669,7 +8669,7 @@
       </c>
       <c r="C199" s="6" t="inlineStr">
         <is>
-          <t>PREMIUM YEMEK SETİ 3'lü</t>
+          <t>PREMIUM 3LÜ SET</t>
         </is>
       </c>
       <c r="D199" s="8" t="inlineStr">
@@ -8679,7 +8679,7 @@
       </c>
       <c r="E199" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F199" s="8" t="inlineStr">
@@ -8751,7 +8751,7 @@
       </c>
       <c r="C201" s="6" t="inlineStr">
         <is>
-          <t>ŞAMPANYA KADEHİ</t>
+          <t>120 CC ŞAMPANYA KADEHİ</t>
         </is>
       </c>
       <c r="D201" s="8" t="inlineStr">
@@ -8761,7 +8761,7 @@
       </c>
       <c r="E201" s="8" t="inlineStr">
         <is>
-          <t>İçecek Bardağı</t>
+          <t>Bardak</t>
         </is>
       </c>
       <c r="F201" s="8" t="inlineStr">
@@ -8792,7 +8792,7 @@
       </c>
       <c r="C202" s="6" t="inlineStr">
         <is>
-          <t>ŞAMPANYA KADEHİ</t>
+          <t>120 CC ŞAMPANYA KADEHİ</t>
         </is>
       </c>
       <c r="D202" s="7" t="inlineStr">
@@ -8802,7 +8802,7 @@
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
-          <t>İçecek Bardağı</t>
+          <t>Bardak</t>
         </is>
       </c>
       <c r="F202" s="7" t="inlineStr">
@@ -8915,7 +8915,7 @@
       </c>
       <c r="C205" s="6" t="inlineStr">
         <is>
-          <t>PRIZMA KAP 200 CC</t>
+          <t>200 CC PRIZMA KAP</t>
         </is>
       </c>
       <c r="D205" s="8" t="inlineStr">
@@ -8997,7 +8997,7 @@
       </c>
       <c r="C207" s="6" t="inlineStr">
         <is>
-          <t>EKO YEMEK SETİ 4'lü</t>
+          <t>EKO 4LÜ SET</t>
         </is>
       </c>
       <c r="D207" s="8" t="inlineStr">
@@ -9007,7 +9007,7 @@
       </c>
       <c r="E207" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F207" s="8" t="inlineStr">
@@ -9079,7 +9079,7 @@
       </c>
       <c r="C209" s="6" t="inlineStr">
         <is>
-          <t>200 cc AYAKLI KASE</t>
+          <t>200 CC AYAKLI KASE</t>
         </is>
       </c>
       <c r="D209" s="8" t="inlineStr">
@@ -9120,7 +9120,7 @@
       </c>
       <c r="C210" s="6" t="inlineStr">
         <is>
-          <t>PRİZMA KAP 60 CC</t>
+          <t>60 CC PRIZMA KAP</t>
         </is>
       </c>
       <c r="D210" s="7" t="inlineStr">
@@ -9858,7 +9858,7 @@
       </c>
       <c r="C228" s="6" t="inlineStr">
         <is>
-          <t>SHOT BARDAK 40 CC</t>
+          <t>SHOT BARDAK 50 CC</t>
         </is>
       </c>
       <c r="D228" s="7" t="inlineStr">
@@ -10186,7 +10186,7 @@
       </c>
       <c r="C236" s="6" t="inlineStr">
         <is>
-          <t>EKO YEMEK SETİ 5'lü</t>
+          <t>EKO 5Lİ SET</t>
         </is>
       </c>
       <c r="D236" s="7" t="inlineStr">
@@ -10196,7 +10196,7 @@
       </c>
       <c r="E236" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F236" s="7" t="inlineStr">
@@ -10268,7 +10268,7 @@
       </c>
       <c r="C238" s="6" t="inlineStr">
         <is>
-          <t>PRİZMA KAP 120 CC</t>
+          <t>120 CC PRIZMA KAP</t>
         </is>
       </c>
       <c r="D238" s="7" t="inlineStr">
@@ -10555,7 +10555,7 @@
       </c>
       <c r="C245" s="6" t="inlineStr">
         <is>
-          <t>SET ESCAJG 2.30 BARKODSUZ DÖKME</t>
+          <t>LUX 3LÜ SET</t>
         </is>
       </c>
       <c r="D245" s="8" t="inlineStr">
@@ -10565,7 +10565,7 @@
       </c>
       <c r="E245" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F245" s="8" t="inlineStr">
@@ -10883,7 +10883,7 @@
       </c>
       <c r="C253" s="6" t="inlineStr">
         <is>
-          <t>PREMIUM YEMEK SETİ 2'lü</t>
+          <t>PREMIUM 2Lİ SET</t>
         </is>
       </c>
       <c r="D253" s="8" t="inlineStr">
@@ -10893,7 +10893,7 @@
       </c>
       <c r="E253" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F253" s="8" t="inlineStr">
@@ -11129,7 +11129,7 @@
       </c>
       <c r="C259" s="6" t="inlineStr">
         <is>
-          <t>PANDA KAŞIK (16*500=8.000)</t>
+          <t>PANDA KAŞIK</t>
         </is>
       </c>
       <c r="D259" s="8" t="inlineStr">
@@ -11170,7 +11170,7 @@
       </c>
       <c r="C260" s="6" t="inlineStr">
         <is>
-          <t>PREMIUM YEMEK SETİ 5'lü</t>
+          <t>PREMIUM 5Lİ SET</t>
         </is>
       </c>
       <c r="D260" s="7" t="inlineStr">
@@ -11180,7 +11180,7 @@
       </c>
       <c r="E260" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F260" s="7" t="inlineStr">
@@ -11293,7 +11293,7 @@
       </c>
       <c r="C263" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">DIAMOND KAŞIK </t>
+          <t>DIAMOND KAŞIK</t>
         </is>
       </c>
       <c r="D263" s="8" t="inlineStr">
@@ -11416,7 +11416,7 @@
       </c>
       <c r="C266" s="6" t="inlineStr">
         <is>
-          <t>PREMIUM SET 3'lü</t>
+          <t>PREMIUM 3LÜ SET</t>
         </is>
       </c>
       <c r="D266" s="7" t="inlineStr">
@@ -11426,7 +11426,7 @@
       </c>
       <c r="E266" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F266" s="7" t="inlineStr">
@@ -11498,7 +11498,7 @@
       </c>
       <c r="C268" s="6" t="inlineStr">
         <is>
-          <t>ŞAMPANYA KADEHİ</t>
+          <t>120 CC ŞAMPANYA KADEHİ</t>
         </is>
       </c>
       <c r="D268" s="7" t="inlineStr">
@@ -11508,7 +11508,7 @@
       </c>
       <c r="E268" s="7" t="inlineStr">
         <is>
-          <t>İçecek Bardağı</t>
+          <t>Bardak</t>
         </is>
       </c>
       <c r="F268" s="7" t="inlineStr">
@@ -11744,7 +11744,7 @@
       </c>
       <c r="C274" s="6" t="inlineStr">
         <is>
-          <t>ŞAMPANYA KADEHİ</t>
+          <t>120 CC ŞAMPANYA KADEHİ</t>
         </is>
       </c>
       <c r="D274" s="7" t="inlineStr">
@@ -11754,7 +11754,7 @@
       </c>
       <c r="E274" s="7" t="inlineStr">
         <is>
-          <t>İçecek Bardağı</t>
+          <t>Bardak</t>
         </is>
       </c>
       <c r="F274" s="7" t="inlineStr">
@@ -11867,7 +11867,7 @@
       </c>
       <c r="C277" s="6" t="inlineStr">
         <is>
-          <t>PRİZMA KAP 200 CC</t>
+          <t>200 CC PRIZMA KAP</t>
         </is>
       </c>
       <c r="D277" s="8" t="inlineStr">
@@ -11908,7 +11908,7 @@
       </c>
       <c r="C278" s="6" t="inlineStr">
         <is>
-          <t>PREMIUM YEMEK SETİ 6'lü</t>
+          <t>PREMIUM 6LI SET</t>
         </is>
       </c>
       <c r="D278" s="7" t="inlineStr">
@@ -11918,7 +11918,7 @@
       </c>
       <c r="E278" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F278" s="7" t="inlineStr">
@@ -11990,7 +11990,7 @@
       </c>
       <c r="C280" s="6" t="inlineStr">
         <is>
-          <t>ŞAMPANYA KADEHİ</t>
+          <t>120 CC ŞAMPANYA KADEHİ</t>
         </is>
       </c>
       <c r="D280" s="7" t="inlineStr">
@@ -12000,7 +12000,7 @@
       </c>
       <c r="E280" s="7" t="inlineStr">
         <is>
-          <t>İçecek Bardağı</t>
+          <t>Bardak</t>
         </is>
       </c>
       <c r="F280" s="7" t="inlineStr">
@@ -12195,7 +12195,7 @@
       </c>
       <c r="C285" s="6" t="inlineStr">
         <is>
-          <t>EKO KAŞIK YEMEK SETİ 2'lü</t>
+          <t>EKO 2Lİ SET</t>
         </is>
       </c>
       <c r="D285" s="8" t="inlineStr">
@@ -12205,7 +12205,7 @@
       </c>
       <c r="E285" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F285" s="8" t="inlineStr">
@@ -12318,7 +12318,7 @@
       </c>
       <c r="C288" s="6" t="inlineStr">
         <is>
-          <t>KAŞIK PLATINUM TEKLİ SET</t>
+          <t>PLATINUM KAŞIK TEKLİ SET</t>
         </is>
       </c>
       <c r="D288" s="7" t="inlineStr">
@@ -12328,7 +12328,7 @@
       </c>
       <c r="E288" s="7" t="inlineStr">
         <is>
-          <t>Kaşık</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F288" s="7" t="inlineStr">
@@ -12441,7 +12441,7 @@
       </c>
       <c r="C291" s="6" t="inlineStr">
         <is>
-          <t>TOSA PREMİUM TATLI KAŞIK</t>
+          <t>PREMIUM TATLI KAŞIK</t>
         </is>
       </c>
       <c r="D291" s="8" t="inlineStr">
@@ -12482,7 +12482,7 @@
       </c>
       <c r="C292" s="6" t="inlineStr">
         <is>
-          <t>SET ESCAJG 3.80 BARKODLU</t>
+          <t>DIAMOND 3LÜ SET</t>
         </is>
       </c>
       <c r="D292" s="7" t="inlineStr">
@@ -12492,7 +12492,7 @@
       </c>
       <c r="E292" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F292" s="7" t="inlineStr">
@@ -12564,7 +12564,7 @@
       </c>
       <c r="C294" s="6" t="inlineStr">
         <is>
-          <t>LÜX CİPS ÇATALI</t>
+          <t>LUX CİPS ÇATALI</t>
         </is>
       </c>
       <c r="D294" s="7" t="inlineStr">
@@ -12933,7 +12933,7 @@
       </c>
       <c r="C303" s="6" t="inlineStr">
         <is>
-          <t>ELİTE YEMEK SETİ 4'lü</t>
+          <t>ELITE 4LÜ SET</t>
         </is>
       </c>
       <c r="D303" s="8" t="inlineStr">
@@ -12943,7 +12943,7 @@
       </c>
       <c r="E303" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F303" s="8" t="inlineStr">
@@ -13015,7 +13015,7 @@
       </c>
       <c r="C305" s="6" t="inlineStr">
         <is>
-          <t>TOSA PREMİUM KAŞIK BEBE</t>
+          <t>PREMIUM KAŞIK</t>
         </is>
       </c>
       <c r="D305" s="8" t="inlineStr">
@@ -13097,7 +13097,7 @@
       </c>
       <c r="C307" s="6" t="inlineStr">
         <is>
-          <t>ÇATAL ELİTE</t>
+          <t>ELITE ÇATAL</t>
         </is>
       </c>
       <c r="D307" s="8" t="inlineStr">
@@ -13138,7 +13138,7 @@
       </c>
       <c r="C308" s="6" t="inlineStr">
         <is>
-          <t>TOSA PREMİUM KAŞIK</t>
+          <t>PREMIUM KAŞIK</t>
         </is>
       </c>
       <c r="D308" s="7" t="inlineStr">
@@ -13179,7 +13179,7 @@
       </c>
       <c r="C309" s="6" t="inlineStr">
         <is>
-          <t>SET ESCAJG 2.80 BARKODLU</t>
+          <t>PREMIUM 3LÜ SET</t>
         </is>
       </c>
       <c r="D309" s="8" t="inlineStr">
@@ -13189,7 +13189,7 @@
       </c>
       <c r="E309" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F309" s="8" t="inlineStr">
@@ -13384,7 +13384,7 @@
       </c>
       <c r="C314" s="6" t="inlineStr">
         <is>
-          <t>KAŞIK PLATINUM TEKLİ SET</t>
+          <t>PLATINUM KAŞIK TEKLİ SET</t>
         </is>
       </c>
       <c r="D314" s="7" t="inlineStr">
@@ -13394,7 +13394,7 @@
       </c>
       <c r="E314" s="7" t="inlineStr">
         <is>
-          <t>Kaşık</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F314" s="7" t="inlineStr">
@@ -13507,7 +13507,7 @@
       </c>
       <c r="C317" s="6" t="inlineStr">
         <is>
-          <t>SET ESCAJG 2.80 BARKODSUZ</t>
+          <t>PREMIUM 3LÜ SET</t>
         </is>
       </c>
       <c r="D317" s="8" t="inlineStr">
@@ -13517,7 +13517,7 @@
       </c>
       <c r="E317" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F317" s="8" t="inlineStr">
@@ -13548,7 +13548,7 @@
       </c>
       <c r="C318" s="6" t="inlineStr">
         <is>
-          <t>KAŞIK ELİTE</t>
+          <t>ELITE KAŞIK</t>
         </is>
       </c>
       <c r="D318" s="7" t="inlineStr">
@@ -13712,7 +13712,7 @@
       </c>
       <c r="C322" s="6" t="inlineStr">
         <is>
-          <t>TEKLİ PREMIUM TATLI KAŞIK SETİ</t>
+          <t>PREMIUM TATLI KAŞIK TEKLİ SET</t>
         </is>
       </c>
       <c r="D322" s="7" t="inlineStr">
@@ -13722,7 +13722,7 @@
       </c>
       <c r="E322" s="7" t="inlineStr">
         <is>
-          <t>Tatlı Kaşığı</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F322" s="7" t="inlineStr">
@@ -13753,7 +13753,7 @@
       </c>
       <c r="C323" s="6" t="inlineStr">
         <is>
-          <t>PİZZA TRİPOT QP</t>
+          <t>PİZZA TRİPOT</t>
         </is>
       </c>
       <c r="D323" s="8" t="inlineStr">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="C328" s="6" t="inlineStr">
         <is>
-          <t>PREMIUM YEMEK SETİ 4'lü</t>
+          <t>PREMIUM 4LÜ SET</t>
         </is>
       </c>
       <c r="D328" s="7" t="inlineStr">
@@ -13968,7 +13968,7 @@
       </c>
       <c r="E328" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F328" s="7" t="inlineStr">
@@ -14040,7 +14040,7 @@
       </c>
       <c r="C330" s="6" t="inlineStr">
         <is>
-          <t>ÇATAL PREMİUM</t>
+          <t>PREMIUM ÇATAL</t>
         </is>
       </c>
       <c r="D330" s="7" t="inlineStr">
@@ -14614,7 +14614,7 @@
       </c>
       <c r="C344" s="6" t="inlineStr">
         <is>
-          <t>PREMIUM KAŞIK TEKLİ YEMEK SETİ</t>
+          <t>PREMIUM KAŞIK TEKLİ SET</t>
         </is>
       </c>
       <c r="D344" s="7" t="inlineStr">
@@ -14624,7 +14624,7 @@
       </c>
       <c r="E344" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F344" s="7" t="inlineStr">
@@ -14737,7 +14737,7 @@
       </c>
       <c r="C347" s="6" t="inlineStr">
         <is>
-          <t>95 MM DONDURMA KAŞIK MİX RENK</t>
+          <t>95 MM DONDURMA KAŞIK</t>
         </is>
       </c>
       <c r="D347" s="8" t="inlineStr">
@@ -14819,7 +14819,7 @@
       </c>
       <c r="C349" s="6" t="inlineStr">
         <is>
-          <t>PREMIUM ÇATAL TEKLİ YEMEK SETİ</t>
+          <t>PREMIUM ÇATAL TEKLİ SET</t>
         </is>
       </c>
       <c r="D349" s="8" t="inlineStr">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="E349" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F349" s="8" t="inlineStr">
@@ -14860,7 +14860,7 @@
       </c>
       <c r="C350" s="6" t="inlineStr">
         <is>
-          <t>ELITE YEMEK SETİ 2'lü</t>
+          <t>ELITE 2Lİ SET</t>
         </is>
       </c>
       <c r="D350" s="7" t="inlineStr">
@@ -14870,7 +14870,7 @@
       </c>
       <c r="E350" s="7" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F350" s="7" t="inlineStr">
@@ -15475,7 +15475,7 @@
       </c>
       <c r="C365" s="6" t="inlineStr">
         <is>
-          <t>TEKLİ PREMIUM KAŞIK SETİ</t>
+          <t>PREMIUM KAŞIK TEKLİ SET</t>
         </is>
       </c>
       <c r="D365" s="8" t="inlineStr">
@@ -15485,7 +15485,7 @@
       </c>
       <c r="E365" s="8" t="inlineStr">
         <is>
-          <t>Kaşık</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F365" s="8" t="inlineStr">
@@ -16910,7 +16910,7 @@
       </c>
       <c r="C400" s="6" t="inlineStr">
         <is>
-          <t>TEKLI PREMIUM KAŞIK SET</t>
+          <t>PREMIUM KAŞIK TEKLİ SET</t>
         </is>
       </c>
       <c r="D400" s="7" t="inlineStr">
@@ -16920,7 +16920,7 @@
       </c>
       <c r="E400" s="7" t="inlineStr">
         <is>
-          <t>Kaşık</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F400" s="7" t="inlineStr">
@@ -17033,7 +17033,7 @@
       </c>
       <c r="C403" s="6" t="inlineStr">
         <is>
-          <t>TEKLI PREMIUM ÇATAL SET</t>
+          <t>PREMIUM ÇATAL TEKLİ SET</t>
         </is>
       </c>
       <c r="D403" s="8" t="inlineStr">
@@ -17043,7 +17043,7 @@
       </c>
       <c r="E403" s="8" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F403" s="8" t="inlineStr">
@@ -17115,7 +17115,7 @@
       </c>
       <c r="C405" s="6" t="inlineStr">
         <is>
-          <t>ŞAMPANYA KADEHİ</t>
+          <t>120 CC ŞAMPANYA KADEHİ</t>
         </is>
       </c>
       <c r="D405" s="8" t="inlineStr">
@@ -17125,7 +17125,7 @@
       </c>
       <c r="E405" s="8" t="inlineStr">
         <is>
-          <t>İçecek Bardağı</t>
+          <t>Bardak</t>
         </is>
       </c>
       <c r="F405" s="8" t="inlineStr">
@@ -17607,7 +17607,7 @@
       </c>
       <c r="C417" s="6" t="inlineStr">
         <is>
-          <t>PANDA KAŞIK (16*500=8.000)</t>
+          <t>PANDA KAŞIK</t>
         </is>
       </c>
       <c r="D417" s="8" t="inlineStr">
@@ -18140,7 +18140,7 @@
       </c>
       <c r="C430" s="6" t="inlineStr">
         <is>
-          <t>ŞAMPANYA KADEHİ</t>
+          <t>120 CC ŞAMPANYA KADEHİ</t>
         </is>
       </c>
       <c r="D430" s="7" t="inlineStr">
@@ -18150,7 +18150,7 @@
       </c>
       <c r="E430" s="7" t="inlineStr">
         <is>
-          <t>İçecek Bardağı</t>
+          <t>Bardak</t>
         </is>
       </c>
       <c r="F430" s="7" t="inlineStr">
@@ -18263,7 +18263,7 @@
       </c>
       <c r="C433" s="6" t="inlineStr">
         <is>
-          <t>ŞAMPANYA KADEHİ</t>
+          <t>120 CC ŞAMPANYA KADEHİ</t>
         </is>
       </c>
       <c r="D433" s="8" t="inlineStr">
@@ -18273,7 +18273,7 @@
       </c>
       <c r="E433" s="8" t="inlineStr">
         <is>
-          <t>İçecek Bardağı</t>
+          <t>Bardak</t>
         </is>
       </c>
       <c r="F433" s="8" t="inlineStr">
@@ -19534,7 +19534,7 @@
       </c>
       <c r="C464" s="6" t="inlineStr">
         <is>
-          <t>BIÇAK PLATINUM TEKLİ SET</t>
+          <t>PLATINUM BIÇAK TEKLİ SET</t>
         </is>
       </c>
       <c r="D464" s="7" t="inlineStr">
@@ -19544,7 +19544,7 @@
       </c>
       <c r="E464" s="7" t="inlineStr">
         <is>
-          <t>Bıçak</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F464" s="7" t="inlineStr">
@@ -19780,7 +19780,7 @@
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>ESTETIK LUX SPOON</t>
+          <t>LUX KAŞIK</t>
         </is>
       </c>
       <c r="D470" t="inlineStr">
@@ -19821,7 +19821,7 @@
       </c>
       <c r="C471" t="inlineStr">
         <is>
-          <t>ESTETIK LUX KNIFE</t>
+          <t>LUX BIÇAK</t>
         </is>
       </c>
       <c r="D471" t="inlineStr">
@@ -19862,7 +19862,7 @@
       </c>
       <c r="C472" t="inlineStr">
         <is>
-          <t>PLA KAŞIK 24'LÜ PAKET</t>
+          <t>PLA DIAMOND KAŞIK</t>
         </is>
       </c>
       <c r="D472" t="inlineStr">
@@ -19903,7 +19903,7 @@
       </c>
       <c r="C473" t="inlineStr">
         <is>
-          <t>PLA ÇATAL 24'LÜ PAKET</t>
+          <t>PLA DIAMOND ÇATAL</t>
         </is>
       </c>
       <c r="D473" t="inlineStr">
@@ -20190,7 +20190,7 @@
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>LÜX BIÇAK</t>
+          <t>LUX BIÇAK</t>
         </is>
       </c>
       <c r="D480" t="inlineStr">
@@ -20559,7 +20559,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>200 CC PRİZMA KAP</t>
+          <t>200 CC PRIZMA KAP</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -20682,7 +20682,7 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>95 MM PLS. DONDURMA KAŞIK</t>
+          <t>95 MM DONDURMA KAŞIK</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
@@ -20723,7 +20723,7 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>200 CC AYAKLI KASE 6'LI PAKET</t>
+          <t>200 CC AYAKLI KASE</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
@@ -20764,7 +20764,7 @@
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>120 CC ŞAMPANYA BARDAK 6'LI PAKET</t>
+          <t>120 CC ŞAMPANYA KADEHİ</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
@@ -21215,7 +21215,7 @@
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>2 OZ SOS KABI</t>
+          <t>2 OZ (60 CC) SOS KABI</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
@@ -21379,7 +21379,7 @@
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>3 LÜ PREMIUM YEMEK SETİ</t>
+          <t>PREMIUM 3LÜ SET</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
@@ -21389,7 +21389,7 @@
       </c>
       <c r="E509" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F509" t="inlineStr">
@@ -21502,7 +21502,7 @@
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>ŞARAP KADEHİ SİYAH</t>
+          <t>ŞARAP KADEHİ</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
@@ -21625,7 +21625,7 @@
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>1 OZ SOS KABI</t>
+          <t>1 OZ (30 CC) SOS KABI</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
@@ -22035,7 +22035,7 @@
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>3 LÜ EKO YEMEK SETİ</t>
+          <t>EKO 3LÜ SET</t>
         </is>
       </c>
       <c r="D525" t="inlineStr">
@@ -22045,7 +22045,7 @@
       </c>
       <c r="E525" t="inlineStr">
         <is>
-          <t>Çatal-Kaşık Set</t>
+          <t>Yemek Seti</t>
         </is>
       </c>
       <c r="F525" t="inlineStr">
@@ -22527,7 +22527,7 @@
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>PANDA KAŞIK (16*500=8.000)</t>
+          <t>PANDA KAŞIK</t>
         </is>
       </c>
       <c r="D537" t="inlineStr">

</xml_diff>

<commit_message>
Apply foam review: fix code 1056, exclude 7 non-product codes, correct foam colors
- code 1056 -> '95 MM DONDURMA KAŞIK' (was mislabeled KÖPÜK ÜRÜNLER; now merges into
  its real product, $25K)
- excluded_stok.json: remove 7 codes (203,209,215,233,822,824,869) — name-similar but
  not company foam products; skipped in all loaders
- taxonomy: apply user's foam color/type fixes (40 types, 26 colors — foam can't be
  transparent, so Şeffaf->Beyaz/Siyah/etc)
- KÖPÜK ÜRÜNLER now $820K with realistic color split (Beyaz/Siyah/Gold/Bej)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RoehW9ESGDK2XkibhR7KNP
</commit_message>
<xml_diff>
--- a/data/taksonomi.xlsx
+++ b/data/taksonomi.xlsx
@@ -1381,7 +1381,7 @@
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F51" s="8" t="inlineStr">
@@ -3062,7 +3062,7 @@
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
@@ -3390,7 +3390,7 @@
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F70" s="8" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F72" s="8" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Bej</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -3800,7 +3800,7 @@
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F80" s="8" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="E90" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F90" s="8" t="inlineStr">
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E91" s="8" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F91" s="8" t="inlineStr">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="E93" s="8" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F93" s="8" t="inlineStr">
@@ -4702,7 +4702,7 @@
       </c>
       <c r="E102" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F102" s="8" t="inlineStr">
@@ -4712,7 +4712,7 @@
       </c>
       <c r="G102" s="7" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
@@ -4825,7 +4825,7 @@
       </c>
       <c r="E105" s="8" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F105" s="8" t="inlineStr">
@@ -4948,7 +4948,7 @@
       </c>
       <c r="E108" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F108" s="8" t="inlineStr">
@@ -4999,7 +4999,7 @@
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H109" s="8" t="n">
@@ -5317,7 +5317,7 @@
       </c>
       <c r="E117" s="8" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F117" s="8" t="inlineStr">
@@ -5358,7 +5358,7 @@
       </c>
       <c r="E118" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F118" s="8" t="inlineStr">
@@ -5399,7 +5399,7 @@
       </c>
       <c r="E119" s="8" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F119" s="8" t="inlineStr">
@@ -5481,7 +5481,7 @@
       </c>
       <c r="E121" s="8" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F121" s="8" t="inlineStr">
@@ -5563,7 +5563,7 @@
       </c>
       <c r="E123" s="8" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F123" s="8" t="inlineStr">
@@ -5573,7 +5573,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H123" s="8" t="n">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="E124" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F124" s="8" t="inlineStr">
@@ -6434,7 +6434,7 @@
       </c>
       <c r="G144" s="7" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H144" s="7" t="n">
@@ -6639,7 +6639,7 @@
       </c>
       <c r="G149" s="8" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H149" s="8" t="n">
@@ -6670,7 +6670,7 @@
       </c>
       <c r="E150" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F150" s="8" t="inlineStr">
@@ -6711,7 +6711,7 @@
       </c>
       <c r="E151" s="8" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F151" s="8" t="inlineStr">
@@ -6721,7 +6721,7 @@
       </c>
       <c r="G151" s="8" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H151" s="8" t="n">
@@ -6793,7 +6793,7 @@
       </c>
       <c r="E153" s="8" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F153" s="8" t="inlineStr">
@@ -6875,7 +6875,7 @@
       </c>
       <c r="E155" s="8" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F155" s="8" t="inlineStr">
@@ -6998,7 +6998,7 @@
       </c>
       <c r="E158" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F158" s="8" t="inlineStr">
@@ -7367,7 +7367,7 @@
       </c>
       <c r="E167" s="8" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F167" s="8" t="inlineStr">
@@ -7490,7 +7490,7 @@
       </c>
       <c r="E170" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F170" s="8" t="inlineStr">
@@ -7500,7 +7500,7 @@
       </c>
       <c r="G170" s="7" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H170" s="7" t="n">
@@ -8023,7 +8023,7 @@
       </c>
       <c r="E183" s="8" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F183" s="8" t="inlineStr">
@@ -8392,7 +8392,7 @@
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F192" s="8" t="inlineStr">
@@ -9171,7 +9171,7 @@
       </c>
       <c r="E211" s="8" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F211" s="8" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="G212" s="7" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H212" s="7" t="n">
@@ -9509,7 +9509,7 @@
       </c>
       <c r="G219" s="8" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H219" s="8" t="n">
@@ -9745,7 +9745,7 @@
       </c>
       <c r="E225" s="8" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F225" s="8" t="inlineStr">
@@ -10739,7 +10739,7 @@
       </c>
       <c r="G249" s="8" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H249" s="8" t="n">
@@ -10934,7 +10934,7 @@
       </c>
       <c r="E254" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F254" s="8" t="inlineStr">
@@ -11016,7 +11016,7 @@
       </c>
       <c r="E256" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F256" s="8" t="inlineStr">
@@ -11057,7 +11057,7 @@
       </c>
       <c r="E257" s="8" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F257" s="8" t="inlineStr">
@@ -12871,7 +12871,7 @@
       </c>
       <c r="G301" s="8" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H301" s="8" t="n">
@@ -13886,7 +13886,7 @@
       </c>
       <c r="E326" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F326" s="7" t="inlineStr">
@@ -14214,7 +14214,7 @@
       </c>
       <c r="E334" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F334" s="8" t="inlineStr">
@@ -14224,7 +14224,7 @@
       </c>
       <c r="G334" s="7" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H334" s="7" t="n">
@@ -14788,7 +14788,7 @@
       </c>
       <c r="E348" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F348" s="8" t="inlineStr">
@@ -14798,7 +14798,7 @@
       </c>
       <c r="G348" s="7" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H348" s="7" t="n">
@@ -15249,7 +15249,7 @@
       </c>
       <c r="G359" s="8" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H359" s="8" t="n">
@@ -15526,7 +15526,7 @@
       </c>
       <c r="E366" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F366" s="8" t="inlineStr">
@@ -15844,7 +15844,7 @@
       </c>
       <c r="C374" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>95 MM DONDURMA KAŞIK</t>
         </is>
       </c>
       <c r="D374" s="8" t="inlineStr">
@@ -15864,7 +15864,7 @@
       </c>
       <c r="G374" s="7" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Turuncu</t>
         </is>
       </c>
       <c r="H374" s="7" t="n">
@@ -16100,7 +16100,7 @@
       </c>
       <c r="E380" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F380" s="7" t="inlineStr">
@@ -16110,7 +16110,7 @@
       </c>
       <c r="G380" s="7" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H380" s="7" t="n">
@@ -16387,7 +16387,7 @@
       </c>
       <c r="E387" s="8" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F387" s="8" t="inlineStr">
@@ -16397,7 +16397,7 @@
       </c>
       <c r="G387" s="8" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H387" s="8" t="n">
@@ -16479,7 +16479,7 @@
       </c>
       <c r="G389" s="8" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H389" s="8" t="n">
@@ -16643,7 +16643,7 @@
       </c>
       <c r="G393" s="8" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H393" s="8" t="n">
@@ -16756,7 +16756,7 @@
       </c>
       <c r="E396" s="7" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Köpük Tabak</t>
         </is>
       </c>
       <c r="F396" s="8" t="inlineStr">
@@ -16766,7 +16766,7 @@
       </c>
       <c r="G396" s="7" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H396" s="7" t="n">
@@ -17258,7 +17258,7 @@
       </c>
       <c r="G408" s="7" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H408" s="7" t="n">
@@ -17340,7 +17340,7 @@
       </c>
       <c r="G410" s="7" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H410" s="7" t="n">
@@ -19595,7 +19595,7 @@
       </c>
       <c r="G465" s="8" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H465" s="8" t="n">
@@ -19636,7 +19636,7 @@
       </c>
       <c r="G466" s="7" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H466" s="7" t="n">

</xml_diff>

<commit_message>
Foam products cannot be transparent: fix remaining Şeffaf->Beyaz (incl code 522)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RoehW9ESGDK2XkibhR7KNP
</commit_message>
<xml_diff>
--- a/data/taksonomi.xlsx
+++ b/data/taksonomi.xlsx
@@ -4507,7 +4507,7 @@
       </c>
       <c r="G97" s="8" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H97" s="8" t="n">
@@ -6147,7 +6147,7 @@
       </c>
       <c r="G137" s="8" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H137" s="8" t="n">
@@ -8730,7 +8730,7 @@
       </c>
       <c r="G200" s="7" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H200" s="7" t="n">
@@ -15700,7 +15700,7 @@
       </c>
       <c r="G370" s="7" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H370" s="7" t="n">
@@ -16602,7 +16602,7 @@
       </c>
       <c r="G392" s="7" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H392" s="7" t="n">
@@ -16725,7 +16725,7 @@
       </c>
       <c r="G395" s="8" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H395" s="8" t="n">
@@ -17422,7 +17422,7 @@
       </c>
       <c r="G412" s="7" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H412" s="7" t="n">
@@ -19513,7 +19513,7 @@
       </c>
       <c r="G463" s="8" t="inlineStr">
         <is>
-          <t>Şeffaf</t>
+          <t>Beyaz</t>
         </is>
       </c>
       <c r="H463" s="8" t="n">

</xml_diff>

<commit_message>
Split KÖPÜK ÜRÜNLER lump into ~20 distinct foam products; exclude 4 more non-products
- Apply user's foam categorization: 56 codes get real TR names + EN translations
  (HB-10 Sandwich Box, MB-3 Meal Box, MOD foam trays, etc)
- excluded_stok += 4 plastic (non-foam) plates (199,585,796,823) -> now 11 excluded
- Products tab: single $800K 'FOAM PRODUCTS' bar replaced by itemized foam products
- Rebuilt: $6.58M, 220 products

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RoehW9ESGDK2XkibhR7KNP
</commit_message>
<xml_diff>
--- a/data/taksonomi.xlsx
+++ b/data/taksonomi.xlsx
@@ -1371,7 +1371,7 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>HB-10 SANDVİÇ KABI</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>HB-10 SANDVİÇ KABI</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MB-3 KAPAKLI 3 GÖZLÜ YEMEK KABI</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
@@ -2601,7 +2601,7 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MB-3 KAPAKLI 3 GÖZLÜ YEMEK KABI</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
@@ -3052,7 +3052,7 @@
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 2 KÜÇÜK KÖPÜK TABAK</t>
         </is>
       </c>
       <c r="D62" s="8" t="inlineStr">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 1 ORTA BOY KÖPÜK TABAK</t>
         </is>
       </c>
       <c r="D70" s="8" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MB-3 KAPAKLI 3 GÖZLÜ YEMEK KABI</t>
         </is>
       </c>
       <c r="D72" s="8" t="inlineStr">
@@ -3790,7 +3790,7 @@
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 2 KÜÇÜK KÖPÜK TABAK</t>
         </is>
       </c>
       <c r="D80" s="8" t="inlineStr">
@@ -4200,7 +4200,7 @@
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 16-A BÜYÜK KÖPÜK TABAK</t>
         </is>
       </c>
       <c r="D90" s="8" t="inlineStr">
@@ -4241,7 +4241,7 @@
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>HB-6 HAMBURGER KABI</t>
         </is>
       </c>
       <c r="D91" s="8" t="inlineStr">
@@ -4323,7 +4323,7 @@
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 16-A BÜYÜK KÖPÜK TABAK</t>
         </is>
       </c>
       <c r="D93" s="8" t="inlineStr">
@@ -4487,7 +4487,7 @@
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MB-3 KAPAKLI 3 GÖZLÜ YEMEK KABI</t>
         </is>
       </c>
       <c r="D97" s="8" t="inlineStr">
@@ -4815,7 +4815,7 @@
       </c>
       <c r="C105" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 1 ORTA BOY KÖPÜK TABAK</t>
         </is>
       </c>
       <c r="D105" s="8" t="inlineStr">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="C108" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MB-2 KAPAKLI 2 GÖZLÜ YEMEK KABI</t>
         </is>
       </c>
       <c r="D108" s="8" t="inlineStr">
@@ -4979,7 +4979,7 @@
       </c>
       <c r="C109" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MB-1 KAPAKLI TEK GÖZLÜ YEMEK KABI</t>
         </is>
       </c>
       <c r="D109" s="8" t="inlineStr">
@@ -5307,7 +5307,7 @@
       </c>
       <c r="C117" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MB-2 KAPAKLI 2 GÖZLÜ YEMEK KABI</t>
         </is>
       </c>
       <c r="D117" s="8" t="inlineStr">
@@ -5348,7 +5348,7 @@
       </c>
       <c r="C118" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>HB-6 HAMBURGER KABI</t>
         </is>
       </c>
       <c r="D118" s="8" t="inlineStr">
@@ -5389,7 +5389,7 @@
       </c>
       <c r="C119" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 16-A BÜYÜK KÖPÜK TABAK</t>
         </is>
       </c>
       <c r="D119" s="8" t="inlineStr">
@@ -5471,7 +5471,7 @@
       </c>
       <c r="C121" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 1 ORTA BOY KÖPÜK TABAK</t>
         </is>
       </c>
       <c r="D121" s="8" t="inlineStr">
@@ -5553,7 +5553,7 @@
       </c>
       <c r="C123" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>HB-6 HAMBURGER KABI</t>
         </is>
       </c>
       <c r="D123" s="8" t="inlineStr">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="C124" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>HB-7 HAMBURGER KABI</t>
         </is>
       </c>
       <c r="D124" s="8" t="inlineStr">
@@ -6127,7 +6127,7 @@
       </c>
       <c r="C137" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MB-1 KAPAKLI TEK GÖZLÜ YEMEK KABI</t>
         </is>
       </c>
       <c r="D137" s="8" t="inlineStr">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C144" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>HB-10 SANDVİÇ KABI</t>
         </is>
       </c>
       <c r="D144" s="8" t="inlineStr">
@@ -6619,7 +6619,7 @@
       </c>
       <c r="C149" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>HB-10 SANDVİÇ KABI</t>
         </is>
       </c>
       <c r="D149" s="8" t="inlineStr">
@@ -6660,7 +6660,7 @@
       </c>
       <c r="C150" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 27-C 4 GÖZLÜ TABİLDOT</t>
         </is>
       </c>
       <c r="D150" s="8" t="inlineStr">
@@ -6783,7 +6783,7 @@
       </c>
       <c r="C153" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 2 KÜÇÜK KÖPÜK TABAK</t>
         </is>
       </c>
       <c r="D153" s="8" t="inlineStr">
@@ -6865,7 +6865,7 @@
       </c>
       <c r="C155" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 1 ORTA BOY KÖPÜK TABAK</t>
         </is>
       </c>
       <c r="D155" s="8" t="inlineStr">
@@ -6988,7 +6988,7 @@
       </c>
       <c r="C158" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 8-C BÜYÜK SIĞ TEPSİ</t>
         </is>
       </c>
       <c r="D158" s="8" t="inlineStr">
@@ -7357,7 +7357,7 @@
       </c>
       <c r="C167" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 2 KÜÇÜK KÖPÜK TABAK</t>
         </is>
       </c>
       <c r="D167" s="8" t="inlineStr">
@@ -7480,7 +7480,7 @@
       </c>
       <c r="C170" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MB-1 KAPAKLI TEK GÖZLÜ YEMEK KABI</t>
         </is>
       </c>
       <c r="D170" s="8" t="inlineStr">
@@ -8013,7 +8013,7 @@
       </c>
       <c r="C183" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MB-1 KAPAKLI TEK GÖZLÜ YEMEK KABI</t>
         </is>
       </c>
       <c r="D183" s="8" t="inlineStr">
@@ -8382,7 +8382,7 @@
       </c>
       <c r="C192" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 16-A BÜYÜK KÖPÜK TABAK</t>
         </is>
       </c>
       <c r="D192" s="8" t="inlineStr">
@@ -9161,7 +9161,7 @@
       </c>
       <c r="C211" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 7 DERİN ORTA BOY KÖPÜK TABAK</t>
         </is>
       </c>
       <c r="D211" s="8" t="inlineStr">
@@ -9202,7 +9202,7 @@
       </c>
       <c r="C212" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MB-1 KAPAKLI TEK GÖZLÜ YEMEK KABI</t>
         </is>
       </c>
       <c r="D212" s="8" t="inlineStr">
@@ -9489,7 +9489,7 @@
       </c>
       <c r="C219" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MB-3 KAPAKLI 3 GÖZLÜ YEMEK KABI</t>
         </is>
       </c>
       <c r="D219" s="8" t="inlineStr">
@@ -9530,7 +9530,7 @@
       </c>
       <c r="C220" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>HB-10 SANDVİÇ KABI</t>
         </is>
       </c>
       <c r="D220" s="8" t="inlineStr">
@@ -9735,7 +9735,7 @@
       </c>
       <c r="C225" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 27-B 5 GÖZLÜ TABİLDOT</t>
         </is>
       </c>
       <c r="D225" s="8" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="C249" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MB-2 KAPAKLI 2 GÖZLÜ YEMEK KABI</t>
         </is>
       </c>
       <c r="D249" s="8" t="inlineStr">
@@ -10924,7 +10924,7 @@
       </c>
       <c r="C254" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 1 ORTA BOY KÖPÜK TABAK</t>
         </is>
       </c>
       <c r="D254" s="8" t="inlineStr">
@@ -11006,7 +11006,7 @@
       </c>
       <c r="C256" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 16-A BÜYÜK KÖPÜK TABAK</t>
         </is>
       </c>
       <c r="D256" s="8" t="inlineStr">
@@ -11047,7 +11047,7 @@
       </c>
       <c r="C257" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>HB-10 SANDVİÇ KABI</t>
         </is>
       </c>
       <c r="D257" s="8" t="inlineStr">
@@ -11662,7 +11662,7 @@
       </c>
       <c r="C272" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MB-1 KAPAKLI TEK GÖZLÜ YEMEK KABI</t>
         </is>
       </c>
       <c r="D272" s="8" t="inlineStr">
@@ -12851,7 +12851,7 @@
       </c>
       <c r="C301" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>HB-9 SANDVİÇ KABI</t>
         </is>
       </c>
       <c r="D301" s="8" t="inlineStr">
@@ -13876,7 +13876,7 @@
       </c>
       <c r="C326" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 7 DERİN ORTA BOY KÖPÜK TABAK</t>
         </is>
       </c>
       <c r="D326" s="7" t="inlineStr">
@@ -14204,7 +14204,7 @@
       </c>
       <c r="C334" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 33-A 17 CM KÜÇÜK YUVARLAK TABAK</t>
         </is>
       </c>
       <c r="D334" s="8" t="inlineStr">
@@ -15229,7 +15229,7 @@
       </c>
       <c r="C359" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 27-B 5 GÖZLÜ TABİLDOT</t>
         </is>
       </c>
       <c r="D359" s="8" t="inlineStr">
@@ -15516,7 +15516,7 @@
       </c>
       <c r="C366" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 2 KÜÇÜK KÖPÜK TABAK</t>
         </is>
       </c>
       <c r="D366" s="8" t="inlineStr">
@@ -16090,7 +16090,7 @@
       </c>
       <c r="C380" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 33-C 23 CM BÜYÜK BOY YUVARLAK TABAK</t>
         </is>
       </c>
       <c r="D380" s="7" t="inlineStr">
@@ -16459,7 +16459,7 @@
       </c>
       <c r="C389" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 122-B DERİN TEPSİ</t>
         </is>
       </c>
       <c r="D389" s="8" t="inlineStr">
@@ -16623,7 +16623,7 @@
       </c>
       <c r="C393" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MB-2 KAPAKLI 2 GÖZLÜ YEMEK KABI</t>
         </is>
       </c>
       <c r="D393" s="8" t="inlineStr">
@@ -16746,7 +16746,7 @@
       </c>
       <c r="C396" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 33-B 20 CM ORTA BOY YUVARLAK TABAK</t>
         </is>
       </c>
       <c r="D396" s="8" t="inlineStr">
@@ -17238,7 +17238,7 @@
       </c>
       <c r="C408" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 14-A PİZZA KUTUSU</t>
         </is>
       </c>
       <c r="D408" s="8" t="inlineStr">
@@ -17320,7 +17320,7 @@
       </c>
       <c r="C410" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>HB-6 HAMBURGER KABI</t>
         </is>
       </c>
       <c r="D410" s="8" t="inlineStr">
@@ -17443,7 +17443,7 @@
       </c>
       <c r="C413" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 7 DERİN ORTA BOY KÖPÜK TABAK</t>
         </is>
       </c>
       <c r="D413" s="8" t="inlineStr">
@@ -19575,7 +19575,7 @@
       </c>
       <c r="C465" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 24 3 GÖZLÜ TABİLDOT</t>
         </is>
       </c>
       <c r="D465" s="8" t="inlineStr">
@@ -19616,7 +19616,7 @@
       </c>
       <c r="C466" s="6" t="inlineStr">
         <is>
-          <t>KÖPÜK ÜRÜNLER</t>
+          <t>MOD 27-C 4 GÖZLÜ TABİLDOT</t>
         </is>
       </c>
       <c r="D466" s="7" t="inlineStr">

</xml_diff>